<commit_message>
Updated Intai bom to indicate camera type
Updated Intai bom to indicate camera type
</commit_message>
<xml_diff>
--- a/BOM/Intai Bom.xlsx
+++ b/BOM/Intai Bom.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="28">
   <si>
     <t>Intai- Camera Based Nozzle Offset Calibration Tool</t>
   </si>
@@ -61,7 +61,7 @@
     <t>n35 or lower</t>
   </si>
   <si>
-    <t>OV9726 Camera module</t>
+    <t>OV9726 Camera module 42deg</t>
   </si>
   <si>
     <t>5v 3mm white led diode</t>
@@ -83,6 +83,9 @@
   </si>
   <si>
     <t>n52</t>
+  </si>
+  <si>
+    <t>OV9726 Camera module 42 deg</t>
   </si>
   <si>
     <t>Floating Base (Switch Version)</t>
@@ -804,7 +807,7 @@
     </row>
     <row r="26">
       <c r="A26" s="21" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B26" s="18">
         <v>1.0</v>
@@ -858,7 +861,7 @@
     </row>
     <row r="31">
       <c r="A31" s="13" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B31" s="14" t="s">
         <v>4</v>
@@ -900,7 +903,7 @@
     </row>
     <row r="35">
       <c r="A35" s="21" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B35" s="18">
         <v>1.0</v>
@@ -934,7 +937,7 @@
     </row>
     <row r="38">
       <c r="A38" s="21" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B38" s="18">
         <v>1.0</v>
@@ -944,7 +947,7 @@
     </row>
     <row r="39">
       <c r="A39" s="21" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B39" s="18">
         <v>1.0</v>

</xml_diff>